<commit_message>
Added co2 concentration to cal in wte (LHV as a function of concentration missing)
</commit_message>
<xml_diff>
--- a/adopt_net0/database/templates/technology_data/Industrial/WasteCaL_data/wasteCaL_sheet.xlsx
+++ b/adopt_net0/database/templates/technology_data/Industrial/WasteCaL_data/wasteCaL_sheet.xlsx
@@ -8,14 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\0954659\PycharmProjects\AdOpT-NET0_luca\adopt_net0\database\templates\technology_data\Industrial\WasteCaL_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32A52545-4038-442F-AD63-957069C41A7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB729878-DDA9-4908-99DE-B6B5C7C46C20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8F88CED2-51E2-4BD6-898E-4BEA1BA4A2AA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{8F88CED2-51E2-4BD6-898E-4BEA1BA4A2AA}"/>
   </bookViews>
   <sheets>
     <sheet name="capex_eur" sheetId="1" r:id="rId1"/>
     <sheet name="emission_factor_waste" sheetId="2" r:id="rId2"/>
     <sheet name="overview_data" sheetId="3" r:id="rId3"/>
+    <sheet name="offdesign_calculations" sheetId="4" r:id="rId4"/>
+    <sheet name="offdesign_results" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -96,7 +98,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="26">
   <si>
     <t>emission_factor_tco2_twaste</t>
   </si>
@@ -126,13 +128,61 @@
   </si>
   <si>
     <t>tCO2/tRDF_including calcination emission</t>
+  </si>
+  <si>
+    <t>lhv_MWh_twaste</t>
+  </si>
+  <si>
+    <t>up flow</t>
+  </si>
+  <si>
+    <t>down flow</t>
+  </si>
+  <si>
+    <t>up conc</t>
+  </si>
+  <si>
+    <t>down conc</t>
+  </si>
+  <si>
+    <t>base</t>
+  </si>
+  <si>
+    <t>net_el_efficiency</t>
+  </si>
+  <si>
+    <t>co2 captured_tph</t>
+  </si>
+  <si>
+    <t>co2 captured_kgps</t>
+  </si>
+  <si>
+    <t>RDF input tRDFptCO2captured</t>
+  </si>
+  <si>
+    <t>RDF input tRDF</t>
+  </si>
+  <si>
+    <t>waste_tph</t>
+  </si>
+  <si>
+    <t>co2_conc</t>
+  </si>
+  <si>
+    <t>rel_el_eff_variation</t>
+  </si>
+  <si>
+    <t>rel_rdf_input_variation</t>
+  </si>
+  <si>
+    <t>relative efficiency variation in per 0,01 of concentration change (BETA) eta_new=eta_design * (1+BETA*(conc[t]-conc_design)) with sign depending on upward/downward change</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -159,6 +209,12 @@
       <color indexed="81"/>
       <name val="Tahoma"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -188,12 +244,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -510,12 +573,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB530849-3AC0-454A-9B3C-7EE06DFB619F}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="3" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B1">
         <v>0.08</v>
       </c>
@@ -523,7 +586,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0</v>
       </c>
@@ -534,7 +597,7 @@
         <v>61956733.735114932</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>21.983665659588002</v>
       </c>
@@ -546,7 +609,7 @@
         <v>187453521.9777776</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>58.616978536727991</v>
       </c>
@@ -557,7 +620,7 @@
         <v>396717686.00048012</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>105.418766019312</v>
       </c>
@@ -568,21 +631,21 @@
         <v>586394103.56009114</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -595,13 +658,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED8393E1-2116-44F4-BC6A-7CAB75645393}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B1">
         <v>0.08</v>
       </c>
@@ -609,15 +672,28 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="6">
         <v>1.1240000000000001</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="6">
         <v>0.89900000000000002</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="5">
+        <f>8.81/3600*1000</f>
+        <v>2.447222222222222</v>
+      </c>
+      <c r="C3" s="5">
+        <f>10.79/3600*1000</f>
+        <v>2.9972222222222218</v>
       </c>
     </row>
   </sheetData>
@@ -629,13 +705,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{360CA07C-9042-4182-B481-990E6A122527}">
   <dimension ref="A2:C6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -646,7 +722,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -657,7 +733,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -668,7 +744,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -679,7 +755,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -688,6 +764,599 @@
       </c>
       <c r="C6" t="s">
         <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF3800F7-44EF-4E95-8339-2B9D4ABCCCA3}">
+  <dimension ref="A1:H23"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="10.42578125" customWidth="1"/>
+    <col min="4" max="4" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="28" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2">
+        <v>69.619621440000003</v>
+      </c>
+      <c r="C2">
+        <v>0.08</v>
+      </c>
+      <c r="D2">
+        <v>16.282494037979998</v>
+      </c>
+      <c r="E2">
+        <v>5.4761578000000002</v>
+      </c>
+      <c r="F2">
+        <v>0.1285572943289566</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3">
+        <v>64.847308679999998</v>
+      </c>
+      <c r="C3">
+        <v>0.08</v>
+      </c>
+      <c r="D3">
+        <v>17.326894819859998</v>
+      </c>
+      <c r="E3">
+        <v>5.8013718799999996</v>
+      </c>
+      <c r="F3">
+        <v>0.12513581457033682</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4">
+        <v>74.391934199999994</v>
+      </c>
+      <c r="C4">
+        <v>0.08</v>
+      </c>
+      <c r="D4">
+        <v>15.233061460769999</v>
+      </c>
+      <c r="E4">
+        <v>5.1487875399999998</v>
+      </c>
+      <c r="F4">
+        <v>0.13047121888388721</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5">
+        <v>69.619621440000003</v>
+      </c>
+      <c r="C5">
+        <v>0.09</v>
+      </c>
+      <c r="D5">
+        <v>18.236537157779999</v>
+      </c>
+      <c r="E5">
+        <v>5.9945676299999997</v>
+      </c>
+      <c r="F5">
+        <v>0.12480663803176834</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6">
+        <v>69.619621440000003</v>
+      </c>
+      <c r="C6">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="D6">
+        <v>14.160805913699999</v>
+      </c>
+      <c r="E6">
+        <v>4.8435427600000001</v>
+      </c>
+      <c r="F6">
+        <v>0.12562956888190682</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E10" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11">
+        <f>B2/$B$2</f>
+        <v>1</v>
+      </c>
+      <c r="C11">
+        <f>C2/$C$2</f>
+        <v>1</v>
+      </c>
+      <c r="D11">
+        <f>D2/1000*3600</f>
+        <v>58.616978536727999</v>
+      </c>
+      <c r="E11">
+        <f>E2/D11</f>
+        <v>9.3422723871186414E-2</v>
+      </c>
+      <c r="F11">
+        <v>0.1285572943289566</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12">
+        <f t="shared" ref="B12:B15" si="0">B3/$B$2</f>
+        <v>0.93145161290322576</v>
+      </c>
+      <c r="C12">
+        <f t="shared" ref="C12:C15" si="1">C3/$C$2</f>
+        <v>1</v>
+      </c>
+      <c r="D12">
+        <f t="shared" ref="D12:D15" si="2">D3/1000*3600</f>
+        <v>62.376821351495991</v>
+      </c>
+      <c r="E12">
+        <f t="shared" ref="E12:E15" si="3">E3/D12</f>
+        <v>9.3005250256485927E-2</v>
+      </c>
+      <c r="F12">
+        <v>0.12513581457033682</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13">
+        <f t="shared" si="0"/>
+        <v>1.068548387096774</v>
+      </c>
+      <c r="C13">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="D13">
+        <f t="shared" si="2"/>
+        <v>54.839021258772</v>
+      </c>
+      <c r="E13">
+        <f t="shared" si="3"/>
+        <v>9.3889121684067336E-2</v>
+      </c>
+      <c r="F13">
+        <v>0.13047121888388721</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14">
+        <f>B5/$B$2</f>
+        <v>1</v>
+      </c>
+      <c r="C14">
+        <f t="shared" si="1"/>
+        <v>1.125</v>
+      </c>
+      <c r="D14">
+        <f t="shared" si="2"/>
+        <v>65.651533768007994</v>
+      </c>
+      <c r="E14">
+        <f t="shared" si="3"/>
+        <v>9.1308874080275548E-2</v>
+      </c>
+      <c r="F14">
+        <v>0.12480663803176834</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="C15">
+        <f t="shared" si="1"/>
+        <v>0.87500000000000011</v>
+      </c>
+      <c r="D15">
+        <f t="shared" si="2"/>
+        <v>50.97890128932</v>
+      </c>
+      <c r="E15">
+        <f t="shared" si="3"/>
+        <v>9.5010732626650676E-2</v>
+      </c>
+      <c r="F15">
+        <v>0.12562956888190682</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D18" t="s">
+        <v>17</v>
+      </c>
+      <c r="E18" t="s">
+        <v>19</v>
+      </c>
+      <c r="F18" t="s">
+        <v>16</v>
+      </c>
+      <c r="G18" t="s">
+        <v>24</v>
+      </c>
+      <c r="H18" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>15</v>
+      </c>
+      <c r="B19">
+        <v>1</v>
+      </c>
+      <c r="C19">
+        <v>0.08</v>
+      </c>
+      <c r="D19">
+        <v>58.616978536727999</v>
+      </c>
+      <c r="E19">
+        <f>E11/$E$11</f>
+        <v>1</v>
+      </c>
+      <c r="F19" s="7">
+        <f>F11/$F$11</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>12</v>
+      </c>
+      <c r="B20">
+        <v>0.93145161290322576</v>
+      </c>
+      <c r="C20">
+        <v>0.08</v>
+      </c>
+      <c r="D20">
+        <v>62.376821351495991</v>
+      </c>
+      <c r="E20">
+        <f t="shared" ref="E20:E23" si="4">E12/$E$11</f>
+        <v>0.99553134829084933</v>
+      </c>
+      <c r="F20" s="1">
+        <f t="shared" ref="F20:F23" si="5">F12/$F$11</f>
+        <v>0.97338556496168327</v>
+      </c>
+      <c r="G20" s="7">
+        <f>($E$19-E20)/(B20-$B$19)</f>
+        <v>-6.518974258055095E-2</v>
+      </c>
+      <c r="H20" s="7">
+        <f>($F$19-F20)/(B20-$B$19)</f>
+        <v>-0.38825764055897322</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>11</v>
+      </c>
+      <c r="B21">
+        <v>1.068548387096774</v>
+      </c>
+      <c r="C21">
+        <v>0.08</v>
+      </c>
+      <c r="D21">
+        <v>54.839021258772</v>
+      </c>
+      <c r="E21">
+        <f t="shared" si="4"/>
+        <v>1.0049923379832513</v>
+      </c>
+      <c r="F21" s="1">
+        <f t="shared" si="5"/>
+        <v>1.0148877165229784</v>
+      </c>
+      <c r="G21" s="7">
+        <f>($E$19-E21)/(B21-$B$19)</f>
+        <v>-7.2829401167430502E-2</v>
+      </c>
+      <c r="H21" s="7">
+        <f>($F$19-F21)/(B21-$B$19)</f>
+        <v>-0.21718551162933217</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>13</v>
+      </c>
+      <c r="B22">
+        <v>1</v>
+      </c>
+      <c r="C22">
+        <v>0.09</v>
+      </c>
+      <c r="D22">
+        <v>65.651533768007994</v>
+      </c>
+      <c r="E22">
+        <f t="shared" si="4"/>
+        <v>0.97737328025432557</v>
+      </c>
+      <c r="F22" s="1">
+        <f t="shared" si="5"/>
+        <v>0.97082502150682359</v>
+      </c>
+      <c r="G22" s="7">
+        <f>($E$19-E22)/(C22-$C$19)</f>
+        <v>2.2626719745674442</v>
+      </c>
+      <c r="H22" s="7">
+        <f>($F$19-F22)/(C22-$C$19)</f>
+        <v>2.917497849317642</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>14</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="D23">
+        <v>50.97890128932</v>
+      </c>
+      <c r="E23">
+        <f t="shared" si="4"/>
+        <v>1.0169980994950849</v>
+      </c>
+      <c r="F23" s="1">
+        <f t="shared" si="5"/>
+        <v>0.97722629849724263</v>
+      </c>
+      <c r="G23" s="7">
+        <f>($E$19-E23)/(C23-$C$19)</f>
+        <v>1.6998099495084915</v>
+      </c>
+      <c r="H23" s="7">
+        <f>(F19-F23)/(C23-C19)</f>
+        <v>-2.2773701502757384</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{808567DB-59C1-42B3-8939-773BE0BF59FD}">
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>0.08</v>
+      </c>
+      <c r="D2">
+        <f>offdesign_calculations!D19</f>
+        <v>58.616978536727999</v>
+      </c>
+      <c r="E2">
+        <f>offdesign_calculations!E19</f>
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <f>offdesign_calculations!F19</f>
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <f>offdesign_calculations!H19</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3">
+        <v>0.93145161290322576</v>
+      </c>
+      <c r="C3">
+        <v>0.08</v>
+      </c>
+      <c r="D3">
+        <f>offdesign_calculations!D20</f>
+        <v>62.376821351495991</v>
+      </c>
+      <c r="E3">
+        <f>offdesign_calculations!E20</f>
+        <v>0.99553134829084933</v>
+      </c>
+      <c r="F3">
+        <f>offdesign_calculations!F20</f>
+        <v>0.97338556496168327</v>
+      </c>
+      <c r="G3">
+        <f>offdesign_calculations!H20</f>
+        <v>-0.38825764055897322</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4">
+        <v>1.068548387096774</v>
+      </c>
+      <c r="C4">
+        <v>0.08</v>
+      </c>
+      <c r="D4">
+        <f>offdesign_calculations!D21</f>
+        <v>54.839021258772</v>
+      </c>
+      <c r="E4">
+        <f>offdesign_calculations!E21</f>
+        <v>1.0049923379832513</v>
+      </c>
+      <c r="F4">
+        <f>offdesign_calculations!F21</f>
+        <v>1.0148877165229784</v>
+      </c>
+      <c r="G4">
+        <f>offdesign_calculations!H21</f>
+        <v>-0.21718551162933217</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>0.09</v>
+      </c>
+      <c r="D5">
+        <f>offdesign_calculations!D22</f>
+        <v>65.651533768007994</v>
+      </c>
+      <c r="E5">
+        <f>offdesign_calculations!E22</f>
+        <v>0.97737328025432557</v>
+      </c>
+      <c r="F5">
+        <f>offdesign_calculations!F22</f>
+        <v>0.97082502150682359</v>
+      </c>
+      <c r="G5">
+        <f>offdesign_calculations!H22</f>
+        <v>2.917497849317642</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="D6">
+        <f>offdesign_calculations!D23</f>
+        <v>50.97890128932</v>
+      </c>
+      <c r="E6">
+        <f>offdesign_calculations!E23</f>
+        <v>1.0169980994950849</v>
+      </c>
+      <c r="F6">
+        <f>offdesign_calculations!F23</f>
+        <v>0.97722629849724263</v>
+      </c>
+      <c r="G6">
+        <f>offdesign_calculations!H23</f>
+        <v>-2.2773701502757384</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated cal bounds, co2 storage costs
</commit_message>
<xml_diff>
--- a/adopt_net0/database/templates/technology_data/Industrial/WasteCaL_data/wasteCaL_sheet.xlsx
+++ b/adopt_net0/database/templates/technology_data/Industrial/WasteCaL_data/wasteCaL_sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\0954659\PycharmProjects\AdOpT-NET0_luca\adopt_net0\database\templates\technology_data\Industrial\WasteCaL_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D893BBC0-F940-479E-BA47-F31EAB3D0A7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DED859B-8FAB-4FFD-95D2-79202286BAB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{8F88CED2-51E2-4BD6-898E-4BEA1BA4A2AA}"/>
+    <workbookView xWindow="28680" yWindow="-75" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{8F88CED2-51E2-4BD6-898E-4BEA1BA4A2AA}"/>
   </bookViews>
   <sheets>
     <sheet name="capex_eur" sheetId="1" r:id="rId1"/>
@@ -98,7 +98,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="29">
   <si>
     <t>emission_factor_tco2_twaste</t>
   </si>
@@ -176,6 +176,15 @@
   </si>
   <si>
     <t>relative efficiency variation in per 0,01 of concentration change (BETA) eta_new=eta_design * (1+BETA*(conc[t]-conc_design)) with sign depending on upward/downward change</t>
+  </si>
+  <si>
+    <t>NOT USEFUL, TH_INPUT DOESN'T CHANGE AND EFFICIENCY CHANGE IS WRONG</t>
+  </si>
+  <si>
+    <t>m</t>
+  </si>
+  <si>
+    <t>b</t>
   </si>
 </sst>
 </file>
@@ -244,7 +253,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -257,6 +266,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -658,21 +668,27 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED8393E1-2116-44F4-BC6A-7CAB75645393}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B1">
         <v>0.08</v>
       </c>
       <c r="C1">
         <v>0.1</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -682,8 +698,16 @@
       <c r="C2" s="6">
         <v>0.89900000000000002</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D2">
+        <f>(C2-B2)/(C1-B1)</f>
+        <v>-11.250000000000002</v>
+      </c>
+      <c r="E2">
+        <f>B2-D2*B1</f>
+        <v>2.024</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -1192,17 +1216,19 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{808567DB-59C1-42B3-8939-773BE0BF59FD}">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="71.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>21</v>
       </c>
@@ -1216,16 +1242,16 @@
         <v>20</v>
       </c>
       <c r="F1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G1" t="s">
         <v>16</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>23</v>
       </c>
-      <c r="H1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -1243,70 +1269,81 @@
         <f>offdesign_calculations!E19</f>
         <v>1</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <f>offdesign_calculations!F19</f>
         <v>1</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <f>offdesign_calculations!H19</f>
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="2">
         <v>0.93145161290322576</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="2">
         <v>0.08</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="2">
         <f>offdesign_calculations!D20</f>
         <v>62.376821351495991</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="2">
         <f>offdesign_calculations!E20</f>
         <v>0.99553134829084933</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="8">
+        <f>offdesign_calculations!G20</f>
+        <v>-6.518974258055095E-2</v>
+      </c>
+      <c r="G3" s="2">
         <f>offdesign_calculations!F20</f>
         <v>0.97338556496168327</v>
       </c>
-      <c r="G3">
+      <c r="H3" s="2">
         <f>offdesign_calculations!H20</f>
         <v>-0.38825764055897322</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="I3" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="2">
         <v>1.068548387096774</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="2">
         <v>0.08</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="2">
         <f>offdesign_calculations!D21</f>
         <v>54.839021258772</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="2">
         <f>offdesign_calculations!E21</f>
         <v>1.0049923379832513</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="8">
+        <f>offdesign_calculations!G21</f>
+        <v>-7.2829401167430502E-2</v>
+      </c>
+      <c r="G4" s="8">
         <f>offdesign_calculations!F21</f>
         <v>1.0148877165229784</v>
       </c>
-      <c r="G4">
+      <c r="H4" s="8">
         <f>offdesign_calculations!H21</f>
         <v>-0.21718551162933217</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -1324,16 +1361,20 @@
         <f>offdesign_calculations!E22</f>
         <v>0.97737328025432557</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="7">
+        <f>offdesign_calculations!G22</f>
+        <v>2.2626719745674442</v>
+      </c>
+      <c r="G5">
         <f>offdesign_calculations!F22</f>
         <v>0.97082502150682359</v>
       </c>
-      <c r="G5">
+      <c r="H5">
         <f>offdesign_calculations!H22</f>
         <v>2.917497849317642</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -1351,16 +1392,21 @@
         <f>offdesign_calculations!E23</f>
         <v>1.0169980994950849</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="7">
+        <f>offdesign_calculations!G23</f>
+        <v>1.6998099495084915</v>
+      </c>
+      <c r="G6">
         <f>offdesign_calculations!F23</f>
         <v>0.97722629849724263</v>
       </c>
-      <c r="G6">
+      <c r="H6">
         <f>offdesign_calculations!H23</f>
         <v>-2.2773701502757384</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Removed interpolation for emission_factor waste based on co2 concentration
</commit_message>
<xml_diff>
--- a/adopt_net0/database/templates/technology_data/Industrial/WasteCaL_data/wasteCaL_sheet.xlsx
+++ b/adopt_net0/database/templates/technology_data/Industrial/WasteCaL_data/wasteCaL_sheet.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\soliscom.uu.nl\geo\SD\Energy and Resources\GazzaniGroup\Luca\Adopt_NET0_Luca\adopt_net0\database\templates\technology_data\Industrial\WasteCaL_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\0954659\PycharmProjects\AdOpT-NET0_luca\adopt_net0\database\templates\technology_data\Industrial\WasteCaL_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25008873-5DE8-482A-9246-D8123BEEAF3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DDF775B-F4D6-4DD1-9659-CD8134C7094F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{8F88CED2-51E2-4BD6-898E-4BEA1BA4A2AA}"/>
   </bookViews>
@@ -267,7 +267,7 @@
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Per cent" xfId="1" builtinId="5"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -283,9 +283,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -323,7 +323,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -429,7 +429,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -571,7 +571,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>

</xml_diff>

<commit_message>
Set piecewise capex of CaL, oxyfuel+mea to be 0 when size is 0. Solves the problem with CAC>co2tax in CaL
</commit_message>
<xml_diff>
--- a/adopt_net0/database/templates/technology_data/Industrial/WasteCaL_data/wasteCaL_sheet.xlsx
+++ b/adopt_net0/database/templates/technology_data/Industrial/WasteCaL_data/wasteCaL_sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\0954659\PycharmProjects\AdOpT-NET0_luca\adopt_net0\database\templates\technology_data\Industrial\WasteCaL_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DDF775B-F4D6-4DD1-9659-CD8134C7094F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44A7FF96-A9A2-42B1-AFB9-6EC9B018234F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{8F88CED2-51E2-4BD6-898E-4BEA1BA4A2AA}"/>
+    <workbookView xWindow="22932" yWindow="-5940" windowWidth="30936" windowHeight="16776" xr2:uid="{8F88CED2-51E2-4BD6-898E-4BEA1BA4A2AA}"/>
   </bookViews>
   <sheets>
     <sheet name="capex_eur" sheetId="1" r:id="rId1"/>
@@ -48,30 +48,6 @@
     <author>Bertoni, L. (Luca)</author>
   </authors>
   <commentList>
-    <comment ref="B2" authorId="0" shapeId="0" xr:uid="{98F8B444-39BC-4ECD-B6AC-F8502D8477D7}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>Bertoni, L. (Luca):</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-I did y=a+bx, computed a and this a is the value reported here</t>
-        </r>
-      </text>
-    </comment>
     <comment ref="B10" authorId="0" shapeId="0" xr:uid="{47898E69-D3BE-4623-8767-126292F5D1D7}">
       <text>
         <r>
@@ -250,7 +226,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -264,6 +240,7 @@
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -580,12 +557,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB530849-3AC0-454A-9B3C-7EE06DFB619F}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="3" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B1">
         <v>0.08</v>
       </c>
@@ -593,18 +570,18 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>0</v>
       </c>
-      <c r="B2" s="2">
-        <v>64292159.343187898</v>
-      </c>
-      <c r="C2" s="2">
-        <v>61956733.735114932</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B2" s="9">
+        <v>0</v>
+      </c>
+      <c r="C2" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>21.983665659588002</v>
       </c>
@@ -616,7 +593,7 @@
         <v>187453521.9777776</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>58.616978536727991</v>
       </c>
@@ -627,7 +604,7 @@
         <v>396717686.00048012</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>105.418766019312</v>
       </c>
@@ -638,21 +615,21 @@
         <v>586394103.56009114</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -666,12 +643,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED8393E1-2116-44F4-BC6A-7CAB75645393}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B1">
         <v>0.08</v>
       </c>
@@ -679,7 +656,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -690,7 +667,7 @@
         <v>0.89900000000000002</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -712,13 +689,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{360CA07C-9042-4182-B481-990E6A122527}">
   <dimension ref="A2:C6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -729,7 +706,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -740,7 +717,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -751,7 +728,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -762,7 +739,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -781,17 +758,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF3800F7-44EF-4E95-8339-2B9D4ABCCCA3}">
   <dimension ref="A1:H23"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="10.42578125" customWidth="1"/>
-    <col min="4" max="4" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="10.44140625" customWidth="1"/>
+    <col min="4" max="4" width="17.5546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="28" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.7109375" customWidth="1"/>
+    <col min="6" max="6" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="D1" t="s">
         <v>18</v>
       </c>
@@ -802,7 +779,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -822,7 +799,7 @@
         <v>0.1285572943289566</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -842,7 +819,7 @@
         <v>0.12513581457033682</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -862,7 +839,7 @@
         <v>0.13047121888388721</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -882,7 +859,7 @@
         <v>0.12480663803176834</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -902,7 +879,7 @@
         <v>0.12562956888190682</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="D10" t="s">
         <v>17</v>
       </c>
@@ -913,7 +890,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -937,7 +914,7 @@
         <v>0.1285572943289566</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -961,7 +938,7 @@
         <v>0.12513581457033682</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -985,7 +962,7 @@
         <v>0.13047121888388721</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -1009,7 +986,7 @@
         <v>0.12480663803176834</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>14</v>
       </c>
@@ -1033,7 +1010,7 @@
         <v>0.12562956888190682</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="D18" t="s">
         <v>17</v>
       </c>
@@ -1050,7 +1027,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>15</v>
       </c>
@@ -1072,7 +1049,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>12</v>
       </c>
@@ -1102,7 +1079,7 @@
         <v>-0.38825764055897322</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>11</v>
       </c>
@@ -1132,7 +1109,7 @@
         <v>-0.21718551162933217</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>13</v>
       </c>
@@ -1162,7 +1139,7 @@
         <v>2.917497849317642</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>14</v>
       </c>
@@ -1200,18 +1177,18 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{808567DB-59C1-42B3-8939-773BE0BF59FD}">
   <dimension ref="A1:I6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="22" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="71.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="71.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>21</v>
       </c>
@@ -1234,7 +1211,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -1261,7 +1238,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>11</v>
       </c>
@@ -1295,7 +1272,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
@@ -1326,7 +1303,7 @@
         <v>-0.21718551162933217</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -1357,7 +1334,7 @@
         <v>2.917497849317642</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>14</v>
       </c>

</xml_diff>

<commit_message>
Added lhv and emission factor as function of time to wasteToEnergy_CaL_ccs.py
</commit_message>
<xml_diff>
--- a/adopt_net0/database/templates/technology_data/Industrial/WasteCaL_data/wasteCaL_sheet.xlsx
+++ b/adopt_net0/database/templates/technology_data/Industrial/WasteCaL_data/wasteCaL_sheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\0954659\PycharmProjects\AdOpT-NET0_luca\adopt_net0\database\templates\technology_data\Industrial\WasteCaL_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44A7FF96-A9A2-42B1-AFB9-6EC9B018234F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EF0CC56-E25D-4C7B-8174-799C5AB3DE4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-5940" windowWidth="30936" windowHeight="16776" xr2:uid="{8F88CED2-51E2-4BD6-898E-4BEA1BA4A2AA}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{8F88CED2-51E2-4BD6-898E-4BEA1BA4A2AA}"/>
   </bookViews>
   <sheets>
     <sheet name="capex_eur" sheetId="1" r:id="rId1"/>
@@ -34,9 +34,6 @@
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -260,9 +257,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -300,7 +297,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -406,7 +403,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -548,7 +545,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -557,12 +554,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB530849-3AC0-454A-9B3C-7EE06DFB619F}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="3" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B1">
         <v>0.08</v>
       </c>
@@ -570,7 +567,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0</v>
       </c>
@@ -581,7 +578,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>21.983665659588002</v>
       </c>
@@ -593,7 +590,7 @@
         <v>187453521.9777776</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>58.616978536727991</v>
       </c>
@@ -604,7 +601,7 @@
         <v>396717686.00048012</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>105.418766019312</v>
       </c>
@@ -615,21 +612,21 @@
         <v>586394103.56009114</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -643,12 +640,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED8393E1-2116-44F4-BC6A-7CAB75645393}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B1">
         <v>0.08</v>
       </c>
@@ -656,18 +653,18 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="6">
-        <v>1.1240000000000001</v>
+        <v>0.89</v>
       </c>
       <c r="C2" s="6">
-        <v>0.89900000000000002</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+        <v>1.04</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -689,13 +686,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{360CA07C-9042-4182-B481-990E6A122527}">
   <dimension ref="A2:C6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -706,7 +703,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -717,7 +714,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -728,7 +725,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -739,7 +736,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -758,17 +755,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF3800F7-44EF-4E95-8339-2B9D4ABCCCA3}">
   <dimension ref="A1:H23"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="10.44140625" customWidth="1"/>
-    <col min="4" max="4" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="10.42578125" customWidth="1"/>
+    <col min="4" max="4" width="17.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="28" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.6640625" customWidth="1"/>
+    <col min="6" max="6" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D1" t="s">
         <v>18</v>
       </c>
@@ -779,7 +776,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -799,7 +796,7 @@
         <v>0.1285572943289566</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -819,7 +816,7 @@
         <v>0.12513581457033682</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -839,7 +836,7 @@
         <v>0.13047121888388721</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -859,7 +856,7 @@
         <v>0.12480663803176834</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -879,7 +876,7 @@
         <v>0.12562956888190682</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D10" t="s">
         <v>17</v>
       </c>
@@ -890,7 +887,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -914,7 +911,7 @@
         <v>0.1285572943289566</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -938,7 +935,7 @@
         <v>0.12513581457033682</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -962,7 +959,7 @@
         <v>0.13047121888388721</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -986,7 +983,7 @@
         <v>0.12480663803176834</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>14</v>
       </c>
@@ -1010,7 +1007,7 @@
         <v>0.12562956888190682</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="D18" t="s">
         <v>17</v>
       </c>
@@ -1027,7 +1024,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>15</v>
       </c>
@@ -1049,7 +1046,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>12</v>
       </c>
@@ -1079,7 +1076,7 @@
         <v>-0.38825764055897322</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>11</v>
       </c>
@@ -1109,7 +1106,7 @@
         <v>-0.21718551162933217</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>13</v>
       </c>
@@ -1139,7 +1136,7 @@
         <v>2.917497849317642</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>14</v>
       </c>
@@ -1177,18 +1174,18 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{808567DB-59C1-42B3-8939-773BE0BF59FD}">
   <dimension ref="A1:I6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="22" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="71.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="71.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>21</v>
       </c>
@@ -1211,7 +1208,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -1238,7 +1235,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>11</v>
       </c>
@@ -1272,7 +1269,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
@@ -1303,7 +1300,7 @@
         <v>-0.21718551162933217</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -1334,7 +1331,7 @@
         <v>2.917497849317642</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>14</v>
       </c>

</xml_diff>

<commit_message>
fixed bp_x of cal capex to be in kmol/h fluegas wte and design concentration to be average if ccs_is_hourly
</commit_message>
<xml_diff>
--- a/adopt_net0/database/templates/technology_data/Industrial/WasteCaL_data/wasteCaL_sheet.xlsx
+++ b/adopt_net0/database/templates/technology_data/Industrial/WasteCaL_data/wasteCaL_sheet.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\0954659\PycharmProjects\AdOpT-NET0_luca\adopt_net0\database\templates\technology_data\Industrial\WasteCaL_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EF0CC56-E25D-4C7B-8174-799C5AB3DE4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC8BECFE-EFD0-49CE-A5E1-EA64904270E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{8F88CED2-51E2-4BD6-898E-4BEA1BA4A2AA}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8F88CED2-51E2-4BD6-898E-4BEA1BA4A2AA}"/>
   </bookViews>
   <sheets>
     <sheet name="capex_eur" sheetId="1" r:id="rId1"/>
     <sheet name="emission_factor_waste" sheetId="2" r:id="rId2"/>
     <sheet name="overview_data" sheetId="3" r:id="rId3"/>
-    <sheet name="offdesign_calculations" sheetId="4" r:id="rId4"/>
-    <sheet name="offdesign_results" sheetId="5" r:id="rId5"/>
+    <sheet name="offdesign_results" sheetId="5" r:id="rId4"/>
+    <sheet name="offdesign_calculations" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +45,7 @@
     <author>Bertoni, L. (Luca)</author>
   </authors>
   <commentList>
-    <comment ref="B10" authorId="0" shapeId="0" xr:uid="{47898E69-D3BE-4623-8767-126292F5D1D7}">
+    <comment ref="A3" authorId="0" shapeId="0" xr:uid="{651CB2DF-8604-42E3-9020-4940AE32B1DD}">
       <text>
         <r>
           <rPr>
@@ -65,7 +65,8 @@
             <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
-I did y=a+bx, computed a and this a is the value reported here</t>
+Data in kmol/h of fle gas from the WtE (so excluding the CaL gases)
+</t>
         </r>
       </text>
     </comment>
@@ -177,6 +178,12 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="9"/>
       <color indexed="81"/>
       <name val="Tahoma"/>
@@ -188,12 +195,6 @@
       <color indexed="81"/>
       <name val="Tahoma"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -223,13 +224,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -238,6 +239,7 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -554,12 +556,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB530849-3AC0-454A-9B3C-7EE06DFB619F}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="3" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B1">
         <v>0.08</v>
       </c>
@@ -567,7 +569,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>0</v>
       </c>
@@ -578,9 +580,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="1">
-        <v>21.983665659588002</v>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="10">
+        <v>3347</v>
       </c>
       <c r="B3" s="3">
         <f>166037113.359973</f>
@@ -590,9 +592,9 @@
         <v>187453521.9777776</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="1">
-        <v>58.616978536727991</v>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="10">
+        <v>8926</v>
       </c>
       <c r="B4">
         <v>335583666.32719898</v>
@@ -601,9 +603,9 @@
         <v>396717686.00048012</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="1">
-        <v>105.418766019312</v>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="10">
+        <v>16066</v>
       </c>
       <c r="B5">
         <v>486368837.80266154</v>
@@ -612,21 +614,20 @@
         <v>586394103.56009114</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -640,12 +641,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED8393E1-2116-44F4-BC6A-7CAB75645393}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="27.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B1">
         <v>0.08</v>
       </c>
@@ -653,7 +654,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -664,7 +665,7 @@
         <v>1.04</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -686,13 +687,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{360CA07C-9042-4182-B481-990E6A122527}">
   <dimension ref="A2:C6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -703,7 +704,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -714,7 +715,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -725,7 +726,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -736,7 +737,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -753,19 +754,26 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF3800F7-44EF-4E95-8339-2B9D4ABCCCA3}">
-  <dimension ref="A1:H23"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{808567DB-59C1-42B3-8939-773BE0BF59FD}">
+  <dimension ref="A1:I6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="10.42578125" customWidth="1"/>
-    <col min="4" max="4" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="28" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.7109375" customWidth="1"/>
+    <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="71.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1" t="s">
+        <v>22</v>
+      </c>
       <c r="D1" t="s">
         <v>18</v>
       </c>
@@ -773,425 +781,189 @@
         <v>20</v>
       </c>
       <c r="F1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>15</v>
       </c>
       <c r="B2">
-        <v>69.619621440000003</v>
+        <v>1</v>
       </c>
       <c r="C2">
         <v>0.08</v>
       </c>
       <c r="D2">
-        <v>16.282494037979998</v>
+        <f>offdesign_calculations!D19</f>
+        <v>58.616978536727999</v>
       </c>
       <c r="E2">
-        <v>5.4761578000000002</v>
-      </c>
-      <c r="F2">
-        <v>0.1285572943289566</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+        <f>offdesign_calculations!E19</f>
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <f>offdesign_calculations!F19</f>
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <f>offdesign_calculations!H19</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="2">
+        <v>0.93145161290322576</v>
+      </c>
+      <c r="C3" s="2">
+        <v>0.08</v>
+      </c>
+      <c r="D3" s="2">
+        <f>offdesign_calculations!D20</f>
+        <v>62.376821351495991</v>
+      </c>
+      <c r="E3" s="2">
+        <f>offdesign_calculations!E20</f>
+        <v>0.99553134829084933</v>
+      </c>
+      <c r="F3" s="8">
+        <f>offdesign_calculations!G20</f>
+        <v>-6.518974258055095E-2</v>
+      </c>
+      <c r="G3" s="2">
+        <f>offdesign_calculations!F20</f>
+        <v>0.97338556496168327</v>
+      </c>
+      <c r="H3" s="2">
+        <f>offdesign_calculations!H20</f>
+        <v>-0.38825764055897322</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B3">
-        <v>64.847308679999998</v>
-      </c>
-      <c r="C3">
+      <c r="B4" s="2">
+        <v>1.068548387096774</v>
+      </c>
+      <c r="C4" s="2">
         <v>0.08</v>
       </c>
-      <c r="D3">
-        <v>17.326894819859998</v>
-      </c>
-      <c r="E3">
-        <v>5.8013718799999996</v>
-      </c>
-      <c r="F3">
-        <v>0.12513581457033682</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4">
-        <v>74.391934199999994</v>
-      </c>
-      <c r="C4">
-        <v>0.08</v>
-      </c>
-      <c r="D4">
-        <v>15.233061460769999</v>
-      </c>
-      <c r="E4">
-        <v>5.1487875399999998</v>
-      </c>
-      <c r="F4">
-        <v>0.13047121888388721</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D4" s="2">
+        <f>offdesign_calculations!D21</f>
+        <v>54.839021258772</v>
+      </c>
+      <c r="E4" s="2">
+        <f>offdesign_calculations!E21</f>
+        <v>1.0049923379832513</v>
+      </c>
+      <c r="F4" s="8">
+        <f>offdesign_calculations!G21</f>
+        <v>-7.2829401167430502E-2</v>
+      </c>
+      <c r="G4" s="8">
+        <f>offdesign_calculations!F21</f>
+        <v>1.0148877165229784</v>
+      </c>
+      <c r="H4" s="8">
+        <f>offdesign_calculations!H21</f>
+        <v>-0.21718551162933217</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>13</v>
       </c>
       <c r="B5">
-        <v>69.619621440000003</v>
+        <v>1</v>
       </c>
       <c r="C5">
         <v>0.09</v>
       </c>
       <c r="D5">
-        <v>18.236537157779999</v>
+        <f>offdesign_calculations!D22</f>
+        <v>65.651533768007994</v>
       </c>
       <c r="E5">
-        <v>5.9945676299999997</v>
-      </c>
-      <c r="F5">
-        <v>0.12480663803176834</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+        <f>offdesign_calculations!E22</f>
+        <v>0.97737328025432557</v>
+      </c>
+      <c r="F5" s="7">
+        <f>offdesign_calculations!G22</f>
+        <v>2.2626719745674442</v>
+      </c>
+      <c r="G5">
+        <f>offdesign_calculations!F22</f>
+        <v>0.97082502150682359</v>
+      </c>
+      <c r="H5">
+        <f>offdesign_calculations!H22</f>
+        <v>2.917497849317642</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>14</v>
       </c>
       <c r="B6">
-        <v>69.619621440000003</v>
+        <v>1</v>
       </c>
       <c r="C6">
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="D6">
-        <v>14.160805913699999</v>
+        <f>offdesign_calculations!D23</f>
+        <v>50.97890128932</v>
       </c>
       <c r="E6">
-        <v>4.8435427600000001</v>
-      </c>
-      <c r="F6">
-        <v>0.12562956888190682</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="D10" t="s">
-        <v>17</v>
-      </c>
-      <c r="E10" t="s">
-        <v>19</v>
-      </c>
-      <c r="F10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11">
-        <f>B2/$B$2</f>
-        <v>1</v>
-      </c>
-      <c r="C11">
-        <f>C2/$C$2</f>
-        <v>1</v>
-      </c>
-      <c r="D11">
-        <f>D2/1000*3600</f>
-        <v>58.616978536727999</v>
-      </c>
-      <c r="E11">
-        <f>E2/D11</f>
-        <v>9.3422723871186414E-2</v>
-      </c>
-      <c r="F11">
-        <v>0.1285572943289566</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B12">
-        <f t="shared" ref="B12:B15" si="0">B3/$B$2</f>
-        <v>0.93145161290322576</v>
-      </c>
-      <c r="C12">
-        <f t="shared" ref="C12:C15" si="1">C3/$C$2</f>
-        <v>1</v>
-      </c>
-      <c r="D12">
-        <f t="shared" ref="D12:D15" si="2">D3/1000*3600</f>
-        <v>62.376821351495991</v>
-      </c>
-      <c r="E12">
-        <f t="shared" ref="E12:E15" si="3">E3/D12</f>
-        <v>9.3005250256485927E-2</v>
-      </c>
-      <c r="F12">
-        <v>0.12513581457033682</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>11</v>
-      </c>
-      <c r="B13">
-        <f t="shared" si="0"/>
-        <v>1.068548387096774</v>
-      </c>
-      <c r="C13">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="D13">
-        <f t="shared" si="2"/>
-        <v>54.839021258772</v>
-      </c>
-      <c r="E13">
-        <f t="shared" si="3"/>
-        <v>9.3889121684067336E-2</v>
-      </c>
-      <c r="F13">
-        <v>0.13047121888388721</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14">
-        <f>B5/$B$2</f>
-        <v>1</v>
-      </c>
-      <c r="C14">
-        <f t="shared" si="1"/>
-        <v>1.125</v>
-      </c>
-      <c r="D14">
-        <f t="shared" si="2"/>
-        <v>65.651533768007994</v>
-      </c>
-      <c r="E14">
-        <f t="shared" si="3"/>
-        <v>9.1308874080275548E-2</v>
-      </c>
-      <c r="F14">
-        <v>0.12480663803176834</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>14</v>
-      </c>
-      <c r="B15">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="C15">
-        <f t="shared" si="1"/>
-        <v>0.87500000000000011</v>
-      </c>
-      <c r="D15">
-        <f t="shared" si="2"/>
-        <v>50.97890128932</v>
-      </c>
-      <c r="E15">
-        <f t="shared" si="3"/>
-        <v>9.5010732626650676E-2</v>
-      </c>
-      <c r="F15">
-        <v>0.12562956888190682</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D18" t="s">
-        <v>17</v>
-      </c>
-      <c r="E18" t="s">
-        <v>19</v>
-      </c>
-      <c r="F18" t="s">
-        <v>16</v>
-      </c>
-      <c r="G18" t="s">
-        <v>24</v>
-      </c>
-      <c r="H18" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>15</v>
-      </c>
-      <c r="B19">
-        <v>1</v>
-      </c>
-      <c r="C19">
-        <v>0.08</v>
-      </c>
-      <c r="D19">
-        <v>58.616978536727999</v>
-      </c>
-      <c r="E19">
-        <f>E11/$E$11</f>
-        <v>1</v>
-      </c>
-      <c r="F19" s="7">
-        <f>F11/$F$11</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>12</v>
-      </c>
-      <c r="B20">
-        <v>0.93145161290322576</v>
-      </c>
-      <c r="C20">
-        <v>0.08</v>
-      </c>
-      <c r="D20">
-        <v>62.376821351495991</v>
-      </c>
-      <c r="E20">
-        <f t="shared" ref="E20:E23" si="4">E12/$E$11</f>
-        <v>0.99553134829084933</v>
-      </c>
-      <c r="F20" s="1">
-        <f t="shared" ref="F20:F23" si="5">F12/$F$11</f>
-        <v>0.97338556496168327</v>
-      </c>
-      <c r="G20" s="7">
-        <f>($E$19-E20)/(B20-$B$19)</f>
-        <v>-6.518974258055095E-2</v>
-      </c>
-      <c r="H20" s="7">
-        <f>($F$19-F20)/(B20-$B$19)</f>
-        <v>-0.38825764055897322</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>11</v>
-      </c>
-      <c r="B21">
-        <v>1.068548387096774</v>
-      </c>
-      <c r="C21">
-        <v>0.08</v>
-      </c>
-      <c r="D21">
-        <v>54.839021258772</v>
-      </c>
-      <c r="E21">
-        <f t="shared" si="4"/>
-        <v>1.0049923379832513</v>
-      </c>
-      <c r="F21" s="1">
-        <f t="shared" si="5"/>
-        <v>1.0148877165229784</v>
-      </c>
-      <c r="G21" s="7">
-        <f>($E$19-E21)/(B21-$B$19)</f>
-        <v>-7.2829401167430502E-2</v>
-      </c>
-      <c r="H21" s="7">
-        <f>($F$19-F21)/(B21-$B$19)</f>
-        <v>-0.21718551162933217</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>13</v>
-      </c>
-      <c r="B22">
-        <v>1</v>
-      </c>
-      <c r="C22">
-        <v>0.09</v>
-      </c>
-      <c r="D22">
-        <v>65.651533768007994</v>
-      </c>
-      <c r="E22">
-        <f t="shared" si="4"/>
-        <v>0.97737328025432557</v>
-      </c>
-      <c r="F22" s="1">
-        <f t="shared" si="5"/>
-        <v>0.97082502150682359</v>
-      </c>
-      <c r="G22" s="7">
-        <f>($E$19-E22)/(C22-$C$19)</f>
-        <v>2.2626719745674442</v>
-      </c>
-      <c r="H22" s="7">
-        <f>($F$19-F22)/(C22-$C$19)</f>
-        <v>2.917497849317642</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>14</v>
-      </c>
-      <c r="B23">
-        <v>1</v>
-      </c>
-      <c r="C23">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="D23">
-        <v>50.97890128932</v>
-      </c>
-      <c r="E23">
-        <f t="shared" si="4"/>
+        <f>offdesign_calculations!E23</f>
         <v>1.0169980994950849</v>
       </c>
-      <c r="F23" s="1">
-        <f t="shared" si="5"/>
+      <c r="F6" s="7">
+        <f>offdesign_calculations!G23</f>
+        <v>1.6998099495084915</v>
+      </c>
+      <c r="G6">
+        <f>offdesign_calculations!F23</f>
         <v>0.97722629849724263</v>
       </c>
-      <c r="G23" s="7">
-        <f>($E$19-E23)/(C23-$C$19)</f>
-        <v>1.6998099495084915</v>
-      </c>
-      <c r="H23" s="7">
-        <f>(F19-F23)/(C23-C19)</f>
+      <c r="H6">
+        <f>offdesign_calculations!H23</f>
         <v>-2.2773701502757384</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{808567DB-59C1-42B3-8939-773BE0BF59FD}">
-  <dimension ref="A1:I6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF3800F7-44EF-4E95-8339-2B9D4ABCCCA3}">
+  <dimension ref="A1:H23"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="71.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="10.44140625" customWidth="1"/>
+    <col min="4" max="4" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="28" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C1" t="s">
-        <v>22</v>
-      </c>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="D1" t="s">
         <v>18</v>
       </c>
@@ -1199,171 +971,400 @@
         <v>20</v>
       </c>
       <c r="F1" t="s">
-        <v>24</v>
-      </c>
-      <c r="G1" t="s">
         <v>16</v>
       </c>
-      <c r="H1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>15</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>69.619621440000003</v>
       </c>
       <c r="C2">
         <v>0.08</v>
       </c>
       <c r="D2">
-        <f>offdesign_calculations!D19</f>
-        <v>58.616978536727999</v>
+        <v>16.282494037979998</v>
       </c>
       <c r="E2">
-        <f>offdesign_calculations!E19</f>
-        <v>1</v>
-      </c>
-      <c r="G2">
-        <f>offdesign_calculations!F19</f>
-        <v>1</v>
-      </c>
-      <c r="H2">
-        <f>offdesign_calculations!H19</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+        <v>5.4761578000000002</v>
+      </c>
+      <c r="F2">
+        <v>0.1285572943289566</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3">
+        <v>64.847308679999998</v>
+      </c>
+      <c r="C3">
+        <v>0.08</v>
+      </c>
+      <c r="D3">
+        <v>17.326894819859998</v>
+      </c>
+      <c r="E3">
+        <v>5.8013718799999996</v>
+      </c>
+      <c r="F3">
+        <v>0.12513581457033682</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="2">
-        <v>0.93145161290322576</v>
-      </c>
-      <c r="C3" s="2">
+      <c r="B4">
+        <v>74.391934199999994</v>
+      </c>
+      <c r="C4">
         <v>0.08</v>
       </c>
-      <c r="D3" s="2">
-        <f>offdesign_calculations!D20</f>
-        <v>62.376821351495991</v>
-      </c>
-      <c r="E3" s="2">
-        <f>offdesign_calculations!E20</f>
-        <v>0.99553134829084933</v>
-      </c>
-      <c r="F3" s="8">
-        <f>offdesign_calculations!G20</f>
-        <v>-6.518974258055095E-2</v>
-      </c>
-      <c r="G3" s="2">
-        <f>offdesign_calculations!F20</f>
-        <v>0.97338556496168327</v>
-      </c>
-      <c r="H3" s="2">
-        <f>offdesign_calculations!H20</f>
-        <v>-0.38825764055897322</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="2">
-        <v>1.068548387096774</v>
-      </c>
-      <c r="C4" s="2">
-        <v>0.08</v>
-      </c>
-      <c r="D4" s="2">
-        <f>offdesign_calculations!D21</f>
-        <v>54.839021258772</v>
-      </c>
-      <c r="E4" s="2">
-        <f>offdesign_calculations!E21</f>
-        <v>1.0049923379832513</v>
-      </c>
-      <c r="F4" s="8">
-        <f>offdesign_calculations!G21</f>
-        <v>-7.2829401167430502E-2</v>
-      </c>
-      <c r="G4" s="8">
-        <f>offdesign_calculations!F21</f>
-        <v>1.0148877165229784</v>
-      </c>
-      <c r="H4" s="8">
-        <f>offdesign_calculations!H21</f>
-        <v>-0.21718551162933217</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="D4">
+        <v>15.233061460769999</v>
+      </c>
+      <c r="E4">
+        <v>5.1487875399999998</v>
+      </c>
+      <c r="F4">
+        <v>0.13047121888388721</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>13</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>69.619621440000003</v>
       </c>
       <c r="C5">
         <v>0.09</v>
       </c>
       <c r="D5">
-        <f>offdesign_calculations!D22</f>
-        <v>65.651533768007994</v>
+        <v>18.236537157779999</v>
       </c>
       <c r="E5">
-        <f>offdesign_calculations!E22</f>
-        <v>0.97737328025432557</v>
-      </c>
-      <c r="F5" s="7">
-        <f>offdesign_calculations!G22</f>
-        <v>2.2626719745674442</v>
-      </c>
-      <c r="G5">
-        <f>offdesign_calculations!F22</f>
-        <v>0.97082502150682359</v>
-      </c>
-      <c r="H5">
-        <f>offdesign_calculations!H22</f>
-        <v>2.917497849317642</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+        <v>5.9945676299999997</v>
+      </c>
+      <c r="F5">
+        <v>0.12480663803176834</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>14</v>
       </c>
       <c r="B6">
-        <v>1</v>
+        <v>69.619621440000003</v>
       </c>
       <c r="C6">
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="D6">
-        <f>offdesign_calculations!D23</f>
+        <v>14.160805913699999</v>
+      </c>
+      <c r="E6">
+        <v>4.8435427600000001</v>
+      </c>
+      <c r="F6">
+        <v>0.12562956888190682</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D10" t="s">
+        <v>17</v>
+      </c>
+      <c r="E10" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11">
+        <f>B2/$B$2</f>
+        <v>1</v>
+      </c>
+      <c r="C11">
+        <f>C2/$C$2</f>
+        <v>1</v>
+      </c>
+      <c r="D11">
+        <f>D2/1000*3600</f>
+        <v>58.616978536727999</v>
+      </c>
+      <c r="E11">
+        <f>E2/D11</f>
+        <v>9.3422723871186414E-2</v>
+      </c>
+      <c r="F11">
+        <v>0.1285572943289566</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12">
+        <f t="shared" ref="B12:B15" si="0">B3/$B$2</f>
+        <v>0.93145161290322576</v>
+      </c>
+      <c r="C12">
+        <f t="shared" ref="C12:C15" si="1">C3/$C$2</f>
+        <v>1</v>
+      </c>
+      <c r="D12">
+        <f t="shared" ref="D12:D15" si="2">D3/1000*3600</f>
+        <v>62.376821351495991</v>
+      </c>
+      <c r="E12">
+        <f t="shared" ref="E12:E15" si="3">E3/D12</f>
+        <v>9.3005250256485927E-2</v>
+      </c>
+      <c r="F12">
+        <v>0.12513581457033682</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13">
+        <f t="shared" si="0"/>
+        <v>1.068548387096774</v>
+      </c>
+      <c r="C13">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="D13">
+        <f t="shared" si="2"/>
+        <v>54.839021258772</v>
+      </c>
+      <c r="E13">
+        <f t="shared" si="3"/>
+        <v>9.3889121684067336E-2</v>
+      </c>
+      <c r="F13">
+        <v>0.13047121888388721</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14">
+        <f>B5/$B$2</f>
+        <v>1</v>
+      </c>
+      <c r="C14">
+        <f t="shared" si="1"/>
+        <v>1.125</v>
+      </c>
+      <c r="D14">
+        <f t="shared" si="2"/>
+        <v>65.651533768007994</v>
+      </c>
+      <c r="E14">
+        <f t="shared" si="3"/>
+        <v>9.1308874080275548E-2</v>
+      </c>
+      <c r="F14">
+        <v>0.12480663803176834</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="C15">
+        <f t="shared" si="1"/>
+        <v>0.87500000000000011</v>
+      </c>
+      <c r="D15">
+        <f t="shared" si="2"/>
         <v>50.97890128932</v>
       </c>
-      <c r="E6">
-        <f>offdesign_calculations!E23</f>
+      <c r="E15">
+        <f t="shared" si="3"/>
+        <v>9.5010732626650676E-2</v>
+      </c>
+      <c r="F15">
+        <v>0.12562956888190682</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D18" t="s">
+        <v>17</v>
+      </c>
+      <c r="E18" t="s">
+        <v>19</v>
+      </c>
+      <c r="F18" t="s">
+        <v>16</v>
+      </c>
+      <c r="G18" t="s">
+        <v>24</v>
+      </c>
+      <c r="H18" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>15</v>
+      </c>
+      <c r="B19">
+        <v>1</v>
+      </c>
+      <c r="C19">
+        <v>0.08</v>
+      </c>
+      <c r="D19">
+        <v>58.616978536727999</v>
+      </c>
+      <c r="E19">
+        <f>E11/$E$11</f>
+        <v>1</v>
+      </c>
+      <c r="F19" s="7">
+        <f>F11/$F$11</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>12</v>
+      </c>
+      <c r="B20">
+        <v>0.93145161290322576</v>
+      </c>
+      <c r="C20">
+        <v>0.08</v>
+      </c>
+      <c r="D20">
+        <v>62.376821351495991</v>
+      </c>
+      <c r="E20">
+        <f t="shared" ref="E20:E23" si="4">E12/$E$11</f>
+        <v>0.99553134829084933</v>
+      </c>
+      <c r="F20" s="1">
+        <f t="shared" ref="F20:F23" si="5">F12/$F$11</f>
+        <v>0.97338556496168327</v>
+      </c>
+      <c r="G20" s="7">
+        <f>($E$19-E20)/(B20-$B$19)</f>
+        <v>-6.518974258055095E-2</v>
+      </c>
+      <c r="H20" s="7">
+        <f>($F$19-F20)/(B20-$B$19)</f>
+        <v>-0.38825764055897322</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>11</v>
+      </c>
+      <c r="B21">
+        <v>1.068548387096774</v>
+      </c>
+      <c r="C21">
+        <v>0.08</v>
+      </c>
+      <c r="D21">
+        <v>54.839021258772</v>
+      </c>
+      <c r="E21">
+        <f t="shared" si="4"/>
+        <v>1.0049923379832513</v>
+      </c>
+      <c r="F21" s="1">
+        <f t="shared" si="5"/>
+        <v>1.0148877165229784</v>
+      </c>
+      <c r="G21" s="7">
+        <f>($E$19-E21)/(B21-$B$19)</f>
+        <v>-7.2829401167430502E-2</v>
+      </c>
+      <c r="H21" s="7">
+        <f>($F$19-F21)/(B21-$B$19)</f>
+        <v>-0.21718551162933217</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>13</v>
+      </c>
+      <c r="B22">
+        <v>1</v>
+      </c>
+      <c r="C22">
+        <v>0.09</v>
+      </c>
+      <c r="D22">
+        <v>65.651533768007994</v>
+      </c>
+      <c r="E22">
+        <f t="shared" si="4"/>
+        <v>0.97737328025432557</v>
+      </c>
+      <c r="F22" s="1">
+        <f t="shared" si="5"/>
+        <v>0.97082502150682359</v>
+      </c>
+      <c r="G22" s="7">
+        <f>($E$19-E22)/(C22-$C$19)</f>
+        <v>2.2626719745674442</v>
+      </c>
+      <c r="H22" s="7">
+        <f>($F$19-F22)/(C22-$C$19)</f>
+        <v>2.917497849317642</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>14</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="D23">
+        <v>50.97890128932</v>
+      </c>
+      <c r="E23">
+        <f t="shared" si="4"/>
         <v>1.0169980994950849</v>
       </c>
-      <c r="F6" s="7">
-        <f>offdesign_calculations!G23</f>
+      <c r="F23" s="1">
+        <f t="shared" si="5"/>
+        <v>0.97722629849724263</v>
+      </c>
+      <c r="G23" s="7">
+        <f>($E$19-E23)/(C23-$C$19)</f>
         <v>1.6998099495084915</v>
       </c>
-      <c r="G6">
-        <f>offdesign_calculations!F23</f>
-        <v>0.97722629849724263</v>
-      </c>
-      <c r="H6">
-        <f>offdesign_calculations!H23</f>
+      <c r="H23" s="7">
+        <f>(F19-F23)/(C23-C19)</f>
         <v>-2.2773701502757384</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated ranges CaL to fit all the possible emitters in the Italy case study
</commit_message>
<xml_diff>
--- a/adopt_net0/database/templates/technology_data/Industrial/WasteCaL_data/wasteCaL_sheet.xlsx
+++ b/adopt_net0/database/templates/technology_data/Industrial/WasteCaL_data/wasteCaL_sheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\0954659\PycharmProjects\AdOpT-NET0_luca\adopt_net0\database\templates\technology_data\Industrial\WasteCaL_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F33E4A2-E051-40B4-AE5D-955BA338D8EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00526A51-CAD1-46A9-AEFF-8CDEA1851BD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{8F88CED2-51E2-4BD6-898E-4BEA1BA4A2AA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8F88CED2-51E2-4BD6-898E-4BEA1BA4A2AA}"/>
   </bookViews>
   <sheets>
     <sheet name="capex_eur" sheetId="1" r:id="rId1"/>
@@ -45,6 +45,56 @@
     <author>Bertoni, L. (Luca)</author>
   </authors>
   <commentList>
+    <comment ref="A5" authorId="0" shapeId="0" xr:uid="{64D304FC-4F89-4E73-99EA-AA114FFF1A61}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Bertoni, L. (Luca):</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+SIZE in kmol of Fluegase from WtE per h
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A6" authorId="0" shapeId="0" xr:uid="{49BFB2C2-848C-4420-9060-357036976EDA}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Bertoni, L. (Luca):</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+EXTRAPOLATED NUMBERS TO ENLARGE THE SIZE RANGE
+</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="B10" authorId="0" shapeId="0" xr:uid="{47898E69-D3BE-4623-8767-126292F5D1D7}">
       <text>
         <r>
@@ -161,7 +211,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -195,6 +245,19 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -223,13 +286,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -237,7 +299,7 @@
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -556,6 +618,7 @@
   <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -571,10 +634,10 @@
       <c r="A2">
         <v>0</v>
       </c>
-      <c r="B2" s="9">
+      <c r="B2">
         <v>0</v>
       </c>
-      <c r="C2" s="9">
+      <c r="C2">
         <v>0</v>
       </c>
     </row>
@@ -582,10 +645,10 @@
       <c r="A3" s="1">
         <v>3347.0983994063113</v>
       </c>
-      <c r="B3" s="4">
+      <c r="B3" s="3">
         <v>166037113.35997301</v>
       </c>
-      <c r="C3" s="4">
+      <c r="C3" s="3">
         <v>187453521.97777799</v>
       </c>
       <c r="E3" s="3"/>
@@ -594,10 +657,10 @@
       <c r="A4" s="1">
         <v>8925.5957317501616</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="3">
         <v>335583666.32719898</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="3">
         <v>396717686.00048</v>
       </c>
     </row>
@@ -612,14 +675,27 @@
         <v>586394103.56009102</v>
       </c>
     </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="8">
+        <v>34000</v>
+      </c>
+      <c r="B6" s="2">
+        <f>_xlfn.FORECAST.LINEAR(A6,B4:B5,A4:A5)</f>
+        <v>865078904.07697272</v>
+      </c>
+      <c r="C6" s="2">
+        <f>_xlfn.FORECAST.LINEAR(A6,C4:C5,A4:A5)</f>
+        <v>1062782915.2832865</v>
+      </c>
+    </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
@@ -653,10 +729,10 @@
       <c r="A2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="6">
+      <c r="B2" s="5">
         <v>0.89</v>
       </c>
-      <c r="C2" s="6">
+      <c r="C2" s="5">
         <v>1.04</v>
       </c>
     </row>
@@ -664,11 +740,11 @@
       <c r="A3" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="5">
+      <c r="B3" s="4">
         <f>8.81/3600*1000</f>
         <v>2.447222222222222</v>
       </c>
-      <c r="C3" s="5">
+      <c r="C3" s="4">
         <f>10.79/3600*1000</f>
         <v>2.9972222222222218</v>
       </c>
@@ -701,10 +777,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B3">
-        <v>1.1240000000000001</v>
+        <v>1.04</v>
       </c>
       <c r="C3" t="s">
         <v>4</v>
@@ -712,7 +788,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4">
         <v>0.89900000000000002</v>
@@ -1037,7 +1113,7 @@
         <f>E11/$E$11</f>
         <v>1</v>
       </c>
-      <c r="F19" s="7">
+      <c r="F19" s="6">
         <f>F11/$F$11</f>
         <v>1</v>
       </c>
@@ -1063,11 +1139,11 @@
         <f t="shared" ref="F20:F23" si="5">F12/$F$11</f>
         <v>0.97338556496168327</v>
       </c>
-      <c r="G20" s="7">
+      <c r="G20" s="6">
         <f>($E$19-E20)/(B20-$B$19)</f>
         <v>-6.518974258055095E-2</v>
       </c>
-      <c r="H20" s="7">
+      <c r="H20" s="6">
         <f>($F$19-F20)/(B20-$B$19)</f>
         <v>-0.38825764055897322</v>
       </c>
@@ -1093,11 +1169,11 @@
         <f t="shared" si="5"/>
         <v>1.0148877165229784</v>
       </c>
-      <c r="G21" s="7">
+      <c r="G21" s="6">
         <f>($E$19-E21)/(B21-$B$19)</f>
         <v>-7.2829401167430502E-2</v>
       </c>
-      <c r="H21" s="7">
+      <c r="H21" s="6">
         <f>($F$19-F21)/(B21-$B$19)</f>
         <v>-0.21718551162933217</v>
       </c>
@@ -1123,11 +1199,11 @@
         <f t="shared" si="5"/>
         <v>0.97082502150682359</v>
       </c>
-      <c r="G22" s="7">
+      <c r="G22" s="6">
         <f>($E$19-E22)/(C22-$C$19)</f>
         <v>2.2626719745674442</v>
       </c>
-      <c r="H22" s="7">
+      <c r="H22" s="6">
         <f>($F$19-F22)/(C22-$C$19)</f>
         <v>2.917497849317642</v>
       </c>
@@ -1153,11 +1229,11 @@
         <f t="shared" si="5"/>
         <v>0.97722629849724263</v>
       </c>
-      <c r="G23" s="7">
+      <c r="G23" s="6">
         <f>($E$19-E23)/(C23-$C$19)</f>
         <v>1.6998099495084915</v>
       </c>
-      <c r="H23" s="7">
+      <c r="H23" s="6">
         <f>(F19-F23)/(C23-C19)</f>
         <v>-2.2773701502757384</v>
       </c>
@@ -1249,7 +1325,7 @@
         <f>offdesign_calculations!E20</f>
         <v>0.99553134829084933</v>
       </c>
-      <c r="F3" s="8">
+      <c r="F3" s="7">
         <f>offdesign_calculations!G20</f>
         <v>-6.518974258055095E-2</v>
       </c>
@@ -1283,15 +1359,15 @@
         <f>offdesign_calculations!E21</f>
         <v>1.0049923379832513</v>
       </c>
-      <c r="F4" s="8">
+      <c r="F4" s="7">
         <f>offdesign_calculations!G21</f>
         <v>-7.2829401167430502E-2</v>
       </c>
-      <c r="G4" s="8">
+      <c r="G4" s="7">
         <f>offdesign_calculations!F21</f>
         <v>1.0148877165229784</v>
       </c>
-      <c r="H4" s="8">
+      <c r="H4" s="7">
         <f>offdesign_calculations!H21</f>
         <v>-0.21718551162933217</v>
       </c>
@@ -1314,7 +1390,7 @@
         <f>offdesign_calculations!E22</f>
         <v>0.97737328025432557</v>
       </c>
-      <c r="F5" s="7">
+      <c r="F5" s="6">
         <f>offdesign_calculations!G22</f>
         <v>2.2626719745674442</v>
       </c>
@@ -1345,7 +1421,7 @@
         <f>offdesign_calculations!E23</f>
         <v>1.0169980994950849</v>
       </c>
-      <c r="F6" s="7">
+      <c r="F6" s="6">
         <f>offdesign_calculations!G23</f>
         <v>1.6998099495084915</v>
       </c>

</xml_diff>

<commit_message>
updated capex cal at size 0 by extrapolating
</commit_message>
<xml_diff>
--- a/adopt_net0/database/templates/technology_data/Industrial/WasteCaL_data/wasteCaL_sheet.xlsx
+++ b/adopt_net0/database/templates/technology_data/Industrial/WasteCaL_data/wasteCaL_sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\0954659\PycharmProjects\AdOpT-NET0_luca\adopt_net0\database\templates\technology_data\Industrial\WasteCaL_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00526A51-CAD1-46A9-AEFF-8CDEA1851BD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{488FB849-ECF7-47ED-8C3D-65A7492CABAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8F88CED2-51E2-4BD6-898E-4BEA1BA4A2AA}"/>
   </bookViews>
@@ -635,10 +635,12 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>0</v>
+        <f>_xlfn.FORECAST.LINEAR(A2,B3:B4,A3:A4)</f>
+        <v>64309181.579637378</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <f>_xlfn.FORECAST.LINEAR(A2,C3:C4,A3:A4)</f>
+        <v>61895023.564156741</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>